<commit_message>
ajuste em formatação de data
</commit_message>
<xml_diff>
--- a/upload/pgto_imp_ret.xlsx
+++ b/upload/pgto_imp_ret.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/doc-netsuite/upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{402CD885-CCF4-4807-8B67-2DCEA4B4FC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{274DF52F-DEDC-48B7-AF79-824F0086D8D1}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{402CD885-CCF4-4807-8B67-2DCEA4B4FC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E283E51D-0B7A-45A6-8F11-F49CF1F33C75}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F4C272B6-AE44-4121-8913-1763B0CD07FD}"/>
   </bookViews>
@@ -186,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>cnpj</t>
   </si>
@@ -227,12 +227,6 @@
     <t>obs</t>
   </si>
   <si>
-    <t>6196001000130</t>
-  </si>
-  <si>
-    <t>5619496000108</t>
-  </si>
-  <si>
     <t>06</t>
   </si>
   <si>
@@ -240,14 +234,31 @@
   </si>
   <si>
     <t>codformtribext</t>
+  </si>
+  <si>
+    <t>00000000000191</t>
+  </si>
+  <si>
+    <t>42253647000175</t>
+  </si>
+  <si>
+    <t>31/10/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -275,11 +286,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,12 +690,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68C7E7DC-222C-4BB2-BAF2-DC57C77B4000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="14.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="15.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5546875" style="3" bestFit="1" customWidth="1"/>
@@ -704,7 +718,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -735,26 +749,26 @@
         <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1">
         <v>1788</v>
       </c>
-      <c r="D2" s="1">
-        <v>45524</v>
-      </c>
-      <c r="E2">
+      <c r="D2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="4">
         <v>12</v>
       </c>
       <c r="F2" s="1">
@@ -773,7 +787,7 @@
         <v>45475</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L2">
         <v>15024</v>
@@ -784,6 +798,9 @@
       <c r="O2">
         <v>10</v>
       </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K7" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Correção no tipo de campo data
</commit_message>
<xml_diff>
--- a/upload/pgto_imp_ret.xlsx
+++ b/upload/pgto_imp_ret.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/doc-netsuite/upload/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{402CD885-CCF4-4807-8B67-2DCEA4B4FC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E283E51D-0B7A-45A6-8F11-F49CF1F33C75}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99DC54A-9EE9-42E4-96E1-F58C987E8D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F4C272B6-AE44-4121-8913-1763B0CD07FD}"/>
+    <workbookView xWindow="0" yWindow="744" windowWidth="23040" windowHeight="12216" xr2:uid="{F4C272B6-AE44-4121-8913-1763B0CD07FD}"/>
   </bookViews>
   <sheets>
     <sheet name="pgtoImpRet" sheetId="1" r:id="rId1"/>
@@ -701,7 +701,7 @@
     <col min="7" max="7" width="9.5546875" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.21875" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.88671875" style="3"/>
-    <col min="10" max="10" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -736,7 +736,7 @@
       <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -783,7 +783,7 @@
       <c r="I2" s="3">
         <v>15</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="5">
         <v>45475</v>
       </c>
       <c r="K2" s="1" t="s">

</xml_diff>